<commit_message>
add tables of assets
</commit_message>
<xml_diff>
--- a/doc/表.xlsx
+++ b/doc/表.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT资产管理系统\ITPM\开发\数据库\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT资产管理系统\ITPM\设计\数据库\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE11AC8E-E0B1-4C26-8E42-76565C77C8A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F648F360-FA96-4DFA-8FFF-18498F4F0399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -398,10 +398,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>关联资产主数据&amp;耗材主数据（均为1：N）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>资产盘点单</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -430,10 +426,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>资产Master数据新增一条；耗材新增/更新一条记录；保存完成后写入出入库履历；根据三级类别更新库存余额</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>sys_dict</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -559,6 +551,14 @@
   </si>
   <si>
     <t>biz_brand_model</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>资产Master数据新增一条或多条；自动生成一条入库登记记录供审批；资产明细写入入库明细中1：N</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>关联资产主数据（1：N）</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -566,7 +566,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -617,6 +617,14 @@
       <family val="2"/>
       <charset val="134"/>
     </font>
+    <font>
+      <strike/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Microsoft YaHei Light"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -659,7 +667,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -671,6 +679,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -957,9 +966,10 @@
     <col min="1" max="1" width="15.375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.625" style="1" customWidth="1"/>
     <col min="3" max="3" width="16.75" style="1" customWidth="1"/>
-    <col min="4" max="4" width="80.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.375" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9" style="1"/>
+    <col min="4" max="4" width="80.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -979,7 +989,7 @@
         <v>18</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -997,7 +1007,7 @@
         <v>19</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1015,7 +1025,7 @@
         <v>19</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1033,7 +1043,7 @@
         <v>19</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1051,7 +1061,7 @@
         <v>19</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1069,7 +1079,7 @@
         <v>19</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1087,7 +1097,7 @@
         <v>19</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1105,7 +1115,7 @@
         <v>19</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1128,7 +1138,7 @@
     </row>
     <row r="10" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>24</v>
@@ -1161,7 +1171,7 @@
         <v>19</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1179,7 +1189,7 @@
         <v>19</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1197,7 +1207,7 @@
         <v>19</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1205,7 +1215,7 @@
         <v>6</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>33</v>
@@ -1215,7 +1225,7 @@
         <v>19</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="15" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1223,7 +1233,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>33</v>
@@ -1233,7 +1243,7 @@
         <v>19</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="16" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1241,7 +1251,7 @@
         <v>32</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>33</v>
@@ -1253,7 +1263,7 @@
         <v>19</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1271,15 +1281,15 @@
         <v>19</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>33</v>
@@ -1289,15 +1299,15 @@
         <v>19</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="19" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>33</v>
@@ -1307,27 +1317,27 @@
         <v>19</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>33</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>19</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1347,7 +1357,7 @@
         <v>19</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1361,13 +1371,13 @@
         <v>43</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>19</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="23" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1384,10 +1394,10 @@
         <v>70</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="24" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1402,10 +1412,10 @@
       </c>
       <c r="D24" s="3"/>
       <c r="E24" s="3" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="25" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1420,10 +1430,10 @@
       </c>
       <c r="D25" s="8"/>
       <c r="E25" s="3" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="26" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1437,53 +1447,53 @@
         <v>57</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="27" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A27" s="8" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>33</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="28" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>43</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="29" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1497,33 +1507,33 @@
         <v>43</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>98</v>
+        <v>129</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>34</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="30" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="D30" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>124</v>
+      <c r="D30" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1537,13 +1547,13 @@
         <v>43</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>34</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="32" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1557,13 +1567,13 @@
         <v>43</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>34</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="33" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1577,13 +1587,13 @@
         <v>43</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>34</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="34" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1597,13 +1607,13 @@
         <v>43</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>34</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="35" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.35">
@@ -1617,18 +1627,18 @@
         <v>43</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>34</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="36" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>82</v>
@@ -1637,61 +1647,61 @@
         <v>43</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>34</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="37" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>43</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>34</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="38" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>43</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>34</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="39" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>43</v>
@@ -1701,12 +1711,12 @@
         <v>34</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="40" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>56</v>
@@ -1719,12 +1729,12 @@
         <v>34</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="41" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>48</v>
@@ -1737,7 +1747,7 @@
         <v>34</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="42" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1755,7 +1765,7 @@
         <v>34</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="43" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1775,7 +1785,7 @@
         <v>34</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="44" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1795,7 +1805,7 @@
         <v>34</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="45" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -1815,7 +1825,7 @@
         <v>34</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>